<commit_message>
Corrida | SFE-RTT | 2026-06-17 11:59:17.947969
</commit_message>
<xml_diff>
--- a/indicadores/SFE-RTT_out.xlsx
+++ b/indicadores/SFE-RTT_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="557">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="559" uniqueCount="559">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -23,7 +23,7 @@
     <t xml:space="preserve">Título</t>
   </si>
   <si>
-    <t xml:space="preserve">Recursos tributarios de la provincia de Santa Fe</t>
+    <t xml:space="preserve">Recursos tributarios totales</t>
   </si>
   <si>
     <t xml:space="preserve">Unidad de medida</t>
@@ -65,6 +65,12 @@
     <t xml:space="preserve">Regresores</t>
   </si>
   <si>
+    <t xml:space="preserve">Alcance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provincia de Santa Fe</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumen del correlograma</t>
   </si>
   <si>
@@ -98,13 +104,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">26/05/2026</t>
+    <t xml:space="preserve">17/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">fleiva</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -2187,9 +2193,13 @@
       <c r="J6" s="1"/>
     </row>
     <row r="7">
-      <c r="A7"/>
+      <c r="A7" t="s">
+        <v>16</v>
+      </c>
       <c r="B7"/>
-      <c r="C7"/>
+      <c r="C7" t="s">
+        <v>17</v>
+      </c>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7"/>
@@ -2200,7 +2210,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B8"/>
       <c r="C8"/>
@@ -2214,12 +2224,12 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.681640615226608</v>
+        <v>0.680782880624759</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -2230,7 +2240,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
@@ -2258,7 +2268,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
@@ -2272,12 +2282,12 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.464633928326507</v>
+        <v>0.463465330551744</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -2300,7 +2310,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
@@ -2314,7 +2324,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B16"/>
       <c r="C16"/>
@@ -2328,7 +2338,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -2342,12 +2352,12 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.000000156773818772033</v>
+        <v>0.00000019156781637269</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -2358,7 +2368,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -2372,12 +2382,12 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.00000795639730978436</v>
+        <v>0.00000872079599574797</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -2520,10 +2530,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B32" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C32"/>
       <c r="D32"/>
@@ -2536,10 +2546,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B33" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C33"/>
       <c r="D33"/>
@@ -2563,66 +2573,66 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="G1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="H1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="I1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="J1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="K1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="L1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="M1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="N1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="O1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="P1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="Q1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="R1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="S1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>146.170313711808</v>
@@ -2675,7 +2685,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>141.069621491034</v>
@@ -2732,7 +2742,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>137.862836962968</v>
@@ -2789,7 +2799,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>139.428551307815</v>
@@ -2846,7 +2856,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>188.667130041942</v>
@@ -2903,7 +2913,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>199.947973988075</v>
@@ -2960,7 +2970,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>157.405573076092</v>
@@ -3017,7 +3027,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>156.742862019058</v>
@@ -3074,7 +3084,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>161.359626045118</v>
@@ -3131,7 +3141,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>144.669140821686</v>
@@ -3188,7 +3198,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>155.792255796975</v>
@@ -3245,7 +3255,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>162.87106765147</v>
@@ -3302,7 +3312,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>163.157648890882</v>
@@ -3361,7 +3371,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>148.811055385272</v>
@@ -3420,7 +3430,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>147.799412884779</v>
@@ -3479,7 +3489,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>145.71636756084</v>
@@ -3538,7 +3548,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>178.402336076903</v>
@@ -3597,7 +3607,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>161.837005539753</v>
@@ -3656,7 +3666,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>158.126078266003</v>
@@ -3715,7 +3725,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>151.843459536923</v>
@@ -3774,7 +3784,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>159.566353798767</v>
@@ -3833,7 +3843,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>168.328769823627</v>
@@ -3892,7 +3902,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>181.779108854629</v>
@@ -3951,7 +3961,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>180.732657438106</v>
@@ -4010,7 +4020,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>155.939061777008</v>
@@ -4069,7 +4079,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>163.327153100048</v>
@@ -4128,7 +4138,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>151.28952862731</v>
@@ -4187,7 +4197,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>155.814849525762</v>
@@ -4246,7 +4256,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>200.517817632934</v>
@@ -4305,7 +4315,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>188.617780928632</v>
@@ -4364,7 +4374,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>159.544958388232</v>
@@ -4423,7 +4433,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>157.987373445332</v>
@@ -4482,7 +4492,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>165.916324346116</v>
@@ -4541,7 +4551,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>169.651369069202</v>
@@ -4600,7 +4610,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>156.305695728212</v>
@@ -4659,7 +4669,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>203.157164304284</v>
@@ -4718,7 +4728,7 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>150.134899971834</v>
@@ -4777,7 +4787,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>152.350616651724</v>
@@ -4836,7 +4846,7 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>135.177504400504</v>
@@ -4895,7 +4905,7 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>136.244432069254</v>
@@ -4954,7 +4964,7 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>180.952609024774</v>
@@ -5013,7 +5023,7 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>163.875730002135</v>
@@ -5072,7 +5082,7 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>162.570833920311</v>
@@ -5131,7 +5141,7 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>151.186191754999</v>
@@ -5190,7 +5200,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>138.518736161037</v>
@@ -5249,7 +5259,7 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>155.359646800687</v>
@@ -5308,7 +5318,7 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B48" s="2" t="n">
         <v>151.233422302441</v>
@@ -5367,7 +5377,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B49" s="2" t="n">
         <v>139.083746280416</v>
@@ -5426,7 +5436,7 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B50" s="2" t="n">
         <v>140.710915465528</v>
@@ -5485,7 +5495,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B51" s="2" t="n">
         <v>145.973567804906</v>
@@ -5544,7 +5554,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B52" s="2" t="n">
         <v>137.028473929348</v>
@@ -5603,7 +5613,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B53" s="2" t="n">
         <v>147.493332802245</v>
@@ -5662,7 +5672,7 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B54" s="2" t="n">
         <v>191.011710601984</v>
@@ -5721,7 +5731,7 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B55" s="2" t="n">
         <v>172.711858994276</v>
@@ -5780,7 +5790,7 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>160.894315375959</v>
@@ -5839,7 +5849,7 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B57" s="2" t="n">
         <v>167.470442407861</v>
@@ -5898,7 +5908,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B58" s="2" t="n">
         <v>150.620345471844</v>
@@ -5957,7 +5967,7 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B59" s="2" t="n">
         <v>149.187506321699</v>
@@ -6016,7 +6026,7 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B60" s="2" t="n">
         <v>171.940521299945</v>
@@ -6075,7 +6085,7 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B61" s="2" t="n">
         <v>154.729863806307</v>
@@ -6134,7 +6144,7 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B62" s="2" t="n">
         <v>152.392369566339</v>
@@ -6193,7 +6203,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B63" s="2" t="n">
         <v>157.229448905268</v>
@@ -6252,7 +6262,7 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>179.523291992702</v>
@@ -6311,7 +6321,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B65" s="2" t="n">
         <v>174.992332310022</v>
@@ -6370,7 +6380,7 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>214.648928462788</v>
@@ -6429,7 +6439,7 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B67" s="2" t="n">
         <v>204.136641665464</v>
@@ -6488,7 +6498,7 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B68" s="2" t="n">
         <v>190.725808969738</v>
@@ -6547,7 +6557,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B69" s="2" t="n">
         <v>191.478182310061</v>
@@ -6606,7 +6616,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B70" s="2" t="n">
         <v>178.761906192944</v>
@@ -6665,7 +6675,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B71" s="2" t="n">
         <v>189.573709443163</v>
@@ -6724,7 +6734,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B72" s="2" t="n">
         <v>190.017313996769</v>
@@ -6783,7 +6793,7 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B73" s="2" t="n">
         <v>178.519454657798</v>
@@ -6842,7 +6852,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B74" s="2" t="n">
         <v>174.590903961019</v>
@@ -6901,7 +6911,7 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B75" s="2" t="n">
         <v>176.645510561789</v>
@@ -6960,7 +6970,7 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B76" s="2" t="n">
         <v>174.057759196389</v>
@@ -7019,7 +7029,7 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B77" s="2" t="n">
         <v>180.615964625086</v>
@@ -7078,7 +7088,7 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B78" s="2" t="n">
         <v>231.362752677219</v>
@@ -7137,7 +7147,7 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B79" s="2" t="n">
         <v>220.329446608989</v>
@@ -7196,7 +7206,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B80" s="2" t="n">
         <v>207.010027268347</v>
@@ -7255,7 +7265,7 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B81" s="2" t="n">
         <v>208.448174603147</v>
@@ -7314,7 +7324,7 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B82" s="2" t="n">
         <v>192.268061786295</v>
@@ -7373,7 +7383,7 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B83" s="2" t="n">
         <v>199.352024444047</v>
@@ -7432,7 +7442,7 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B84" s="2" t="n">
         <v>201.926866534716</v>
@@ -7491,7 +7501,7 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B85" s="2" t="n">
         <v>191.278971964862</v>
@@ -7550,7 +7560,7 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B86" s="2" t="n">
         <v>175.638691804137</v>
@@ -7609,7 +7619,7 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B87" s="2" t="n">
         <v>177.487930017691</v>
@@ -7668,7 +7678,7 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B88" s="2" t="n">
         <v>171.915597454502</v>
@@ -7727,7 +7737,7 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B89" s="2" t="n">
         <v>178.374541409015</v>
@@ -7786,7 +7796,7 @@
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B90" s="2" t="n">
         <v>227.223060151939</v>
@@ -7845,7 +7855,7 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B91" s="2" t="n">
         <v>220.94639693754</v>
@@ -7904,7 +7914,7 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B92" s="2" t="n">
         <v>199.742260114853</v>
@@ -7963,7 +7973,7 @@
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B93" s="2" t="n">
         <v>204.603944032525</v>
@@ -8022,7 +8032,7 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B94" s="2" t="n">
         <v>189.415703092519</v>
@@ -8081,7 +8091,7 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B95" s="2" t="n">
         <v>197.27960985569</v>
@@ -8140,7 +8150,7 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B96" s="2" t="n">
         <v>205.056210646535</v>
@@ -8199,7 +8209,7 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B97" s="2" t="n">
         <v>224.780475787984</v>
@@ -8258,7 +8268,7 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B98" s="2" t="n">
         <v>210.765742755235</v>
@@ -8317,7 +8327,7 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B99" s="2" t="n">
         <v>207.791521703906</v>
@@ -8376,7 +8386,7 @@
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B100" s="2" t="n">
         <v>193.684700283605</v>
@@ -8435,7 +8445,7 @@
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B101" s="2" t="n">
         <v>211.008442093289</v>
@@ -8494,7 +8504,7 @@
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B102" s="2" t="n">
         <v>206.969383778428</v>
@@ -8553,7 +8563,7 @@
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B103" s="2" t="n">
         <v>209.12853836621</v>
@@ -8612,7 +8622,7 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B104" s="2" t="n">
         <v>216.129591735927</v>
@@ -8671,7 +8681,7 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B105" s="2" t="n">
         <v>202.087320892804</v>
@@ -8730,7 +8740,7 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B106" s="2" t="n">
         <v>201.816399907871</v>
@@ -8789,7 +8799,7 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B107" s="2" t="n">
         <v>207.613045752276</v>
@@ -8848,7 +8858,7 @@
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B108" s="2" t="n">
         <v>207.720478636926</v>
@@ -8907,7 +8917,7 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B109" s="2" t="n">
         <v>197.18930717241</v>
@@ -8966,7 +8976,7 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B110" s="2" t="n">
         <v>204.04971612926</v>
@@ -9025,7 +9035,7 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B111" s="2" t="n">
         <v>194.030311667106</v>
@@ -9084,7 +9094,7 @@
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B112" s="2" t="n">
         <v>201.187616263748</v>
@@ -9143,7 +9153,7 @@
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B113" s="2" t="n">
         <v>198.832083266279</v>
@@ -9202,7 +9212,7 @@
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B114" s="2" t="n">
         <v>227.952136643138</v>
@@ -9261,7 +9271,7 @@
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B115" s="2" t="n">
         <v>209.746611620456</v>
@@ -9320,7 +9330,7 @@
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B116" s="2" t="n">
         <v>187.395427679135</v>
@@ -9379,7 +9389,7 @@
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B117" s="2" t="n">
         <v>205.312599840642</v>
@@ -9438,7 +9448,7 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B118" s="2" t="n">
         <v>170.252144812846</v>
@@ -9497,7 +9507,7 @@
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B119" s="2" t="n">
         <v>168.19816853489</v>
@@ -9556,7 +9566,7 @@
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B120" s="2" t="n">
         <v>155.479702437859</v>
@@ -9615,7 +9625,7 @@
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B121" s="2" t="n">
         <v>104.713664700098</v>
@@ -9674,7 +9684,7 @@
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B122" s="2" t="n">
         <v>178.270356550411</v>
@@ -9733,7 +9743,7 @@
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B123" s="2" t="n">
         <v>172.294485252959</v>
@@ -9792,7 +9802,7 @@
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B124" s="2" t="n">
         <v>158.973252606958</v>
@@ -9851,7 +9861,7 @@
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B125" s="2" t="n">
         <v>145.736905638761</v>
@@ -9910,7 +9920,7 @@
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B126" s="2" t="n">
         <v>145.555653410911</v>
@@ -9969,7 +9979,7 @@
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B127" s="2" t="n">
         <v>136.805077189649</v>
@@ -10028,7 +10038,7 @@
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B128" s="2" t="n">
         <v>138.18166651147</v>
@@ -10087,7 +10097,7 @@
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B129" s="2" t="n">
         <v>129.436689858629</v>
@@ -10146,7 +10156,7 @@
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B130" s="2" t="n">
         <v>125.699604188077</v>
@@ -10205,7 +10215,7 @@
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B131" s="2" t="n">
         <v>133.264558913449</v>
@@ -10264,7 +10274,7 @@
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B132" s="2" t="n">
         <v>133.916321911938</v>
@@ -10323,7 +10333,7 @@
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B133" s="2" t="n">
         <v>127.060437426622</v>
@@ -10382,7 +10392,7 @@
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B134" s="2" t="n">
         <v>141.310666303849</v>
@@ -10441,7 +10451,7 @@
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B135" s="2" t="n">
         <v>111.560704972489</v>
@@ -10500,7 +10510,7 @@
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B136" s="2" t="n">
         <v>108.824944164063</v>
@@ -10559,7 +10569,7 @@
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B137" s="2" t="n">
         <v>125.537527793496</v>
@@ -10618,7 +10628,7 @@
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B138" s="2" t="n">
         <v>177.532634859878</v>
@@ -10677,7 +10687,7 @@
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B139" s="2" t="n">
         <v>148.346783107403</v>
@@ -10736,7 +10746,7 @@
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B140" s="2" t="n">
         <v>138.501922937188</v>
@@ -10795,7 +10805,7 @@
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B141" s="2" t="n">
         <v>153.822487424438</v>
@@ -10854,7 +10864,7 @@
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B142" s="2" t="n">
         <v>162.558083629551</v>
@@ -10913,7 +10923,7 @@
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B143" s="2" t="n">
         <v>165.869345625873</v>
@@ -10972,7 +10982,7 @@
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B144" s="2" t="n">
         <v>178.923733782982</v>
@@ -11031,7 +11041,7 @@
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B145" s="2" t="n">
         <v>181.069919106976</v>
@@ -11090,7 +11100,7 @@
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B146" s="2" t="n">
         <v>164.060213058262</v>
@@ -11149,7 +11159,7 @@
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B147" s="2" t="n">
         <v>157.863854771553</v>
@@ -11208,7 +11218,7 @@
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B148" s="2" t="n">
         <v>179.158033597095</v>
@@ -11267,7 +11277,7 @@
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B149" s="2" t="n">
         <v>168.02780220227</v>
@@ -11326,7 +11336,7 @@
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B150" s="2" t="n">
         <v>288.13656825188</v>
@@ -11385,7 +11395,7 @@
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B151" s="2" t="n">
         <v>233.724229434968</v>
@@ -11444,7 +11454,7 @@
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B152" s="2" t="n">
         <v>191.877312805501</v>
@@ -11503,7 +11513,7 @@
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B153" s="2" t="n">
         <v>209.105744949749</v>
@@ -11562,7 +11572,7 @@
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B154" s="2" t="n">
         <v>189.900145369112</v>
@@ -11621,7 +11631,7 @@
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B155" s="2" t="n">
         <v>201.136424236631</v>
@@ -11680,7 +11690,7 @@
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B156" s="2" t="n">
         <v>192.9953918995</v>
@@ -11739,7 +11749,7 @@
     </row>
     <row r="157">
       <c r="A157" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B157" s="2" t="n">
         <v>183.579307022865</v>
@@ -11798,7 +11808,7 @@
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B158" s="2" t="n">
         <v>201.725041605403</v>
@@ -11857,7 +11867,7 @@
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B159" s="2" t="n">
         <v>201.046512042623</v>
@@ -11916,7 +11926,7 @@
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B160" s="2" t="n">
         <v>181.638226411986</v>
@@ -11975,7 +11985,7 @@
     </row>
     <row r="161">
       <c r="A161" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B161" s="2" t="n">
         <v>204.637737423437</v>
@@ -12034,7 +12044,7 @@
     </row>
     <row r="162">
       <c r="A162" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B162" s="2" t="n">
         <v>267.431040182923</v>
@@ -12093,7 +12103,7 @@
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B163" s="2" t="n">
         <v>255.307031234999</v>
@@ -12152,7 +12162,7 @@
     </row>
     <row r="164">
       <c r="A164" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B164" s="2" t="n">
         <v>216.042308734758</v>
@@ -12211,7 +12221,7 @@
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B165" s="2" t="n">
         <v>215.264485745364</v>
@@ -12270,7 +12280,7 @@
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B166" s="2" t="n">
         <v>218.710840377079</v>
@@ -12329,7 +12339,7 @@
     </row>
     <row r="167">
       <c r="A167" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B167" s="2" t="n">
         <v>217.572791119282</v>
@@ -12388,7 +12398,7 @@
     </row>
     <row r="168">
       <c r="A168" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B168" s="2" t="n">
         <v>220.953036834014</v>
@@ -12447,7 +12457,7 @@
     </row>
     <row r="169">
       <c r="A169" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B169" s="2" t="n">
         <v>226.401091208185</v>
@@ -12506,7 +12516,7 @@
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B170" s="2" t="n">
         <v>210.935378317033</v>
@@ -12565,7 +12575,7 @@
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B171" s="2" t="n">
         <v>228.561560318637</v>
@@ -12624,7 +12634,7 @@
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B172" s="2" t="n">
         <v>201.184103546968</v>
@@ -12683,7 +12693,7 @@
     </row>
     <row r="173">
       <c r="A173" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B173" s="2" t="n">
         <v>193.902698060345</v>
@@ -12742,7 +12752,7 @@
     </row>
     <row r="174">
       <c r="A174" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B174" s="2" t="n">
         <v>282.307705541931</v>
@@ -12801,7 +12811,7 @@
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B175" s="2" t="n">
         <v>289.006822499009</v>
@@ -12860,7 +12870,7 @@
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B176" s="2" t="n">
         <v>244.079687757216</v>
@@ -12919,7 +12929,7 @@
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B177" s="2" t="n">
         <v>248.038481507858</v>
@@ -12978,7 +12988,7 @@
     </row>
     <row r="178">
       <c r="A178" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B178" s="2" t="n">
         <v>241.904047209842</v>
@@ -13037,7 +13047,7 @@
     </row>
     <row r="179">
       <c r="A179" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B179" s="2" t="n">
         <v>249.014271112847</v>
@@ -13096,7 +13106,7 @@
     </row>
     <row r="180">
       <c r="A180" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B180" s="2" t="n">
         <v>252.839897989163</v>
@@ -13155,7 +13165,7 @@
     </row>
     <row r="181">
       <c r="A181" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B181" s="2" t="n">
         <v>244.040947482251</v>
@@ -13214,7 +13224,7 @@
     </row>
     <row r="182">
       <c r="A182" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B182" s="2" t="n">
         <v>248.920146194045</v>
@@ -13273,7 +13283,7 @@
     </row>
     <row r="183">
       <c r="A183" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B183" s="2" t="n">
         <v>250.446165942311</v>
@@ -13332,7 +13342,7 @@
     </row>
     <row r="184">
       <c r="A184" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B184" s="2" t="n">
         <v>225.959466519764</v>
@@ -13391,7 +13401,7 @@
     </row>
     <row r="185">
       <c r="A185" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B185" s="2" t="n">
         <v>220.762398872638</v>
@@ -13450,7 +13460,7 @@
     </row>
     <row r="186">
       <c r="A186" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B186" s="2" t="n">
         <v>319.669380845044</v>
@@ -13509,7 +13519,7 @@
     </row>
     <row r="187">
       <c r="A187" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B187" s="2" t="n">
         <v>322.575969853798</v>
@@ -13568,7 +13578,7 @@
     </row>
     <row r="188">
       <c r="A188" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B188" s="2" t="n">
         <v>281.905910006439</v>
@@ -13627,7 +13637,7 @@
     </row>
     <row r="189">
       <c r="A189" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B189" s="2" t="n">
         <v>294.41457018889</v>
@@ -13686,7 +13696,7 @@
     </row>
     <row r="190">
       <c r="A190" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B190" s="2" t="n">
         <v>273.701430047225</v>
@@ -13745,7 +13755,7 @@
     </row>
     <row r="191">
       <c r="A191" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B191" s="2" t="n">
         <v>281.08726019336</v>
@@ -13804,7 +13814,7 @@
     </row>
     <row r="192">
       <c r="A192" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B192" s="2" t="n">
         <v>291.904746416023</v>
@@ -13863,7 +13873,7 @@
     </row>
     <row r="193">
       <c r="A193" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B193" s="2" t="n">
         <v>295.454910680978</v>
@@ -13922,7 +13932,7 @@
     </row>
     <row r="194">
       <c r="A194" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B194" s="2" t="n">
         <v>294.153359184623</v>
@@ -13981,7 +13991,7 @@
     </row>
     <row r="195">
       <c r="A195" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B195" s="2" t="n">
         <v>297.192190348533</v>
@@ -14040,7 +14050,7 @@
     </row>
     <row r="196">
       <c r="A196" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B196" s="2" t="n">
         <v>236.988298966396</v>
@@ -14099,7 +14109,7 @@
     </row>
     <row r="197">
       <c r="A197" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B197" s="2" t="n">
         <v>267.130646529735</v>
@@ -14158,7 +14168,7 @@
     </row>
     <row r="198">
       <c r="A198" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B198" s="2" t="n">
         <v>335.23442066469</v>
@@ -14217,7 +14227,7 @@
     </row>
     <row r="199">
       <c r="A199" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B199" s="2" t="n">
         <v>333.136098046109</v>
@@ -14276,7 +14286,7 @@
     </row>
     <row r="200">
       <c r="A200" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B200" s="2" t="n">
         <v>307.028429608668</v>
@@ -14335,7 +14345,7 @@
     </row>
     <row r="201">
       <c r="A201" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B201" s="2" t="n">
         <v>301.793637451609</v>
@@ -14394,7 +14404,7 @@
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B202" s="2" t="n">
         <v>285.3959334707</v>
@@ -14453,7 +14463,7 @@
     </row>
     <row r="203">
       <c r="A203" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B203" s="2" t="n">
         <v>293.005720917596</v>
@@ -14512,7 +14522,7 @@
     </row>
     <row r="204">
       <c r="A204" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B204" s="2" t="n">
         <v>269.594988286548</v>
@@ -14571,7 +14581,7 @@
     </row>
     <row r="205">
       <c r="A205" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B205" s="2" t="n">
         <v>279.655165786659</v>
@@ -14630,7 +14640,7 @@
     </row>
     <row r="206">
       <c r="A206" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B206" s="2" t="n">
         <v>263.91268318791</v>
@@ -14689,7 +14699,7 @@
     </row>
     <row r="207">
       <c r="A207" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B207" s="2" t="n">
         <v>275.371596793728</v>
@@ -14748,7 +14758,7 @@
     </row>
     <row r="208">
       <c r="A208" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B208" s="2" t="n">
         <v>239.165029361958</v>
@@ -14807,7 +14817,7 @@
     </row>
     <row r="209">
       <c r="A209" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B209" s="2" t="n">
         <v>252.261113290537</v>
@@ -14866,7 +14876,7 @@
     </row>
     <row r="210">
       <c r="A210" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B210" s="2" t="n">
         <v>314.664853160642</v>
@@ -14925,7 +14935,7 @@
     </row>
     <row r="211">
       <c r="A211" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B211" s="2" t="n">
         <v>319.203845066844</v>
@@ -14984,7 +14994,7 @@
     </row>
     <row r="212">
       <c r="A212" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B212" s="2" t="n">
         <v>285.550203550335</v>
@@ -15043,7 +15053,7 @@
     </row>
     <row r="213">
       <c r="A213" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B213" s="2" t="n">
         <v>285.851088444828</v>
@@ -15102,7 +15112,7 @@
     </row>
     <row r="214">
       <c r="A214" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B214" s="2" t="n">
         <v>288.626995198861</v>
@@ -15161,7 +15171,7 @@
     </row>
     <row r="215">
       <c r="A215" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B215" s="2" t="n">
         <v>292.037525878689</v>
@@ -15220,7 +15230,7 @@
     </row>
     <row r="216">
       <c r="A216" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B216" s="2" t="n">
         <v>276.835570894392</v>
@@ -15279,7 +15289,7 @@
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B217" s="2" t="n">
         <v>280.66445065934</v>
@@ -15338,7 +15348,7 @@
     </row>
     <row r="218">
       <c r="A218" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B218" s="2" t="n">
         <v>260.384068231554</v>
@@ -15397,7 +15407,7 @@
     </row>
     <row r="219">
       <c r="A219" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B219" s="2" t="n">
         <v>286.486665463863</v>
@@ -15456,7 +15466,7 @@
     </row>
     <row r="220">
       <c r="A220" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B220" s="2" t="n">
         <v>275.89283255791</v>
@@ -15515,7 +15525,7 @@
     </row>
     <row r="221">
       <c r="A221" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B221" s="2" t="n">
         <v>296.979909804655</v>
@@ -15574,7 +15584,7 @@
     </row>
     <row r="222">
       <c r="A222" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B222" s="2" t="n">
         <v>393.469296191174</v>
@@ -15633,7 +15643,7 @@
     </row>
     <row r="223">
       <c r="A223" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B223" s="2" t="n">
         <v>372.545715857446</v>
@@ -15692,7 +15702,7 @@
     </row>
     <row r="224">
       <c r="A224" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B224" s="2" t="n">
         <v>329.971512555091</v>
@@ -15751,7 +15761,7 @@
     </row>
     <row r="225">
       <c r="A225" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B225" s="2" t="n">
         <v>327.456150363785</v>
@@ -15810,7 +15820,7 @@
     </row>
     <row r="226">
       <c r="A226" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B226" s="2" t="n">
         <v>317.499608053578</v>
@@ -15869,7 +15879,7 @@
     </row>
     <row r="227">
       <c r="A227" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B227" s="2" t="n">
         <v>306.732876053814</v>
@@ -15928,7 +15938,7 @@
     </row>
     <row r="228">
       <c r="A228" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B228" s="2" t="n">
         <v>318.994408664709</v>
@@ -15987,7 +15997,7 @@
     </row>
     <row r="229">
       <c r="A229" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B229" s="2" t="n">
         <v>332.331245586257</v>
@@ -16046,7 +16056,7 @@
     </row>
     <row r="230">
       <c r="A230" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B230" s="2" t="n">
         <v>316.165990249722</v>
@@ -16105,7 +16115,7 @@
     </row>
     <row r="231">
       <c r="A231" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B231" s="2" t="n">
         <v>321.265387221039</v>
@@ -16164,7 +16174,7 @@
     </row>
     <row r="232">
       <c r="A232" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B232" s="2" t="n">
         <v>303.052886377943</v>
@@ -16223,7 +16233,7 @@
     </row>
     <row r="233">
       <c r="A233" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B233" s="2" t="n">
         <v>310.919001810919</v>
@@ -16282,7 +16292,7 @@
     </row>
     <row r="234">
       <c r="A234" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B234" s="2" t="n">
         <v>418.243272328397</v>
@@ -16341,7 +16351,7 @@
     </row>
     <row r="235">
       <c r="A235" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B235" s="2" t="n">
         <v>399.674057657919</v>
@@ -16400,7 +16410,7 @@
     </row>
     <row r="236">
       <c r="A236" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B236" s="2" t="n">
         <v>357.730394107374</v>
@@ -16459,7 +16469,7 @@
     </row>
     <row r="237">
       <c r="A237" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B237" s="2" t="n">
         <v>348.272476592456</v>
@@ -16518,7 +16528,7 @@
     </row>
     <row r="238">
       <c r="A238" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B238" s="2" t="n">
         <v>354.023760178911</v>
@@ -16577,7 +16587,7 @@
     </row>
     <row r="239">
       <c r="A239" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B239" s="2" t="n">
         <v>342.573413584462</v>
@@ -16636,7 +16646,7 @@
     </row>
     <row r="240">
       <c r="A240" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B240" s="2" t="n">
         <v>357.579386826068</v>
@@ -16695,7 +16705,7 @@
     </row>
     <row r="241">
       <c r="A241" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B241" s="2" t="n">
         <v>336.539166732192</v>
@@ -16754,7 +16764,7 @@
     </row>
     <row r="242">
       <c r="A242" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B242" s="2" t="n">
         <v>337.605901271908</v>
@@ -16813,7 +16823,7 @@
     </row>
     <row r="243">
       <c r="A243" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B243" s="2" t="n">
         <v>337.777878039721</v>
@@ -16872,7 +16882,7 @@
     </row>
     <row r="244">
       <c r="A244" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B244" s="2" t="n">
         <v>317.002406633981</v>
@@ -16931,7 +16941,7 @@
     </row>
     <row r="245">
       <c r="A245" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B245" s="2" t="n">
         <v>300.178032546421</v>
@@ -16990,7 +17000,7 @@
     </row>
     <row r="246">
       <c r="A246" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B246" s="2" t="n">
         <v>408.116883532572</v>
@@ -17049,7 +17059,7 @@
     </row>
     <row r="247">
       <c r="A247" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B247" s="2" t="n">
         <v>393.051992177606</v>
@@ -17108,7 +17118,7 @@
     </row>
     <row r="248">
       <c r="A248" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B248" s="2" t="n">
         <v>343.700490758097</v>
@@ -17167,7 +17177,7 @@
     </row>
     <row r="249">
       <c r="A249" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B249" s="2" t="n">
         <v>357.431724940695</v>
@@ -17226,7 +17236,7 @@
     </row>
     <row r="250">
       <c r="A250" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B250" s="2" t="n">
         <v>337.856511248639</v>
@@ -17285,7 +17295,7 @@
     </row>
     <row r="251">
       <c r="A251" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B251" s="2" t="n">
         <v>366.092968665438</v>
@@ -17344,7 +17354,7 @@
     </row>
     <row r="252">
       <c r="A252" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B252" s="2" t="n">
         <v>368.412915078779</v>
@@ -17403,7 +17413,7 @@
     </row>
     <row r="253">
       <c r="A253" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B253" s="2" t="n">
         <v>363.535557663137</v>
@@ -17462,7 +17472,7 @@
     </row>
     <row r="254">
       <c r="A254" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B254" s="2" t="n">
         <v>350.043891497069</v>
@@ -17521,7 +17531,7 @@
     </row>
     <row r="255">
       <c r="A255" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B255" s="2" t="n">
         <v>375.921044287891</v>
@@ -17580,7 +17590,7 @@
     </row>
     <row r="256">
       <c r="A256" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B256" s="2" t="n">
         <v>341.102274771443</v>
@@ -17639,7 +17649,7 @@
     </row>
     <row r="257">
       <c r="A257" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B257" s="2" t="n">
         <v>353.641256186117</v>
@@ -17698,7 +17708,7 @@
     </row>
     <row r="258">
       <c r="A258" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B258" s="2" t="n">
         <v>439.069857617465</v>
@@ -17757,7 +17767,7 @@
     </row>
     <row r="259">
       <c r="A259" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B259" s="2" t="n">
         <v>434.208800234975</v>
@@ -17816,7 +17826,7 @@
     </row>
     <row r="260">
       <c r="A260" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B260" s="2" t="n">
         <v>380.151213528173</v>
@@ -17875,7 +17885,7 @@
     </row>
     <row r="261">
       <c r="A261" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B261" s="2" t="n">
         <v>387.620881045035</v>
@@ -17934,7 +17944,7 @@
     </row>
     <row r="262">
       <c r="A262" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B262" s="2" t="n">
         <v>371.264038772031</v>
@@ -17993,7 +18003,7 @@
     </row>
     <row r="263">
       <c r="A263" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B263" s="2" t="n">
         <v>371.812275950725</v>
@@ -18052,7 +18062,7 @@
     </row>
     <row r="264">
       <c r="A264" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B264" s="2" t="n">
         <v>377.60322348967</v>
@@ -18111,7 +18121,7 @@
     </row>
     <row r="265">
       <c r="A265" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B265" s="2" t="n">
         <v>369.846316453117</v>
@@ -18170,7 +18180,7 @@
     </row>
     <row r="266">
       <c r="A266" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B266" s="2" t="n">
         <v>379.060183114088</v>
@@ -18229,7 +18239,7 @@
     </row>
     <row r="267">
       <c r="A267" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B267" s="2" t="n">
         <v>389.340099355369</v>
@@ -18288,7 +18298,7 @@
     </row>
     <row r="268">
       <c r="A268" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B268" s="2" t="n">
         <v>320.821060877805</v>
@@ -18347,7 +18357,7 @@
     </row>
     <row r="269">
       <c r="A269" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B269" s="2" t="n">
         <v>345.52467434589</v>
@@ -18406,7 +18416,7 @@
     </row>
     <row r="270">
       <c r="A270" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B270" s="2" t="n">
         <v>413.450230754435</v>
@@ -18465,7 +18475,7 @@
     </row>
     <row r="271">
       <c r="A271" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B271" s="2" t="n">
         <v>413.229703120197</v>
@@ -18524,7 +18534,7 @@
     </row>
     <row r="272">
       <c r="A272" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B272" s="2" t="n">
         <v>366.725400312327</v>
@@ -18583,7 +18593,7 @@
     </row>
     <row r="273">
       <c r="A273" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B273" s="2" t="n">
         <v>368.630114040458</v>
@@ -18642,7 +18652,7 @@
     </row>
     <row r="274">
       <c r="A274" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B274" s="2" t="n">
         <v>378.032032216345</v>
@@ -18701,7 +18711,7 @@
     </row>
     <row r="275">
       <c r="A275" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B275" s="2" t="n">
         <v>370.653161014162</v>
@@ -18760,7 +18770,7 @@
     </row>
     <row r="276">
       <c r="A276" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B276" s="2" t="n">
         <v>368.660379021458</v>
@@ -18819,7 +18829,7 @@
     </row>
     <row r="277">
       <c r="A277" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B277" s="2" t="n">
         <v>375.412539666912</v>
@@ -18878,7 +18888,7 @@
     </row>
     <row r="278">
       <c r="A278" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B278" s="2" t="n">
         <v>361.94883183059</v>
@@ -18937,7 +18947,7 @@
     </row>
     <row r="279">
       <c r="A279" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B279" s="2" t="n">
         <v>381.453981804347</v>
@@ -18996,7 +19006,7 @@
     </row>
     <row r="280">
       <c r="A280" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B280" s="2" t="n">
         <v>329.488146830178</v>
@@ -19055,7 +19065,7 @@
     </row>
     <row r="281">
       <c r="A281" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B281" s="2" t="n">
         <v>375.164983133172</v>
@@ -19114,7 +19124,7 @@
     </row>
     <row r="282">
       <c r="A282" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B282" s="2" t="n">
         <v>438.262114954461</v>
@@ -19173,7 +19183,7 @@
     </row>
     <row r="283">
       <c r="A283" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B283" s="2" t="n">
         <v>446.374601752146</v>
@@ -19232,7 +19242,7 @@
     </row>
     <row r="284">
       <c r="A284" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B284" s="2" t="n">
         <v>394.274442744795</v>
@@ -19291,7 +19301,7 @@
     </row>
     <row r="285">
       <c r="A285" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B285" s="2" t="n">
         <v>394.860693793777</v>
@@ -19350,7 +19360,7 @@
     </row>
     <row r="286">
       <c r="A286" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B286" s="2" t="n">
         <v>388.416969054151</v>
@@ -19409,7 +19419,7 @@
     </row>
     <row r="287">
       <c r="A287" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B287" s="2" t="n">
         <v>390.356051284665</v>
@@ -19468,7 +19478,7 @@
     </row>
     <row r="288">
       <c r="A288" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B288" s="2" t="n">
         <v>386.489278738235</v>
@@ -19527,7 +19537,7 @@
     </row>
     <row r="289">
       <c r="A289" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B289" s="2" t="n">
         <v>456.923059200996</v>
@@ -19586,7 +19596,7 @@
     </row>
     <row r="290">
       <c r="A290" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B290" s="2" t="n">
         <v>437.846257349914</v>
@@ -19645,7 +19655,7 @@
     </row>
     <row r="291">
       <c r="A291" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B291" s="2" t="n">
         <v>418.060970734171</v>
@@ -19704,7 +19714,7 @@
     </row>
     <row r="292">
       <c r="A292" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B292" s="2" t="n">
         <v>377.550949733574</v>
@@ -19763,7 +19773,7 @@
     </row>
     <row r="293">
       <c r="A293" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B293" s="2" t="n">
         <v>382.135240400365</v>
@@ -19822,7 +19832,7 @@
     </row>
     <row r="294">
       <c r="A294" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B294" s="2" t="n">
         <v>417.84450291248</v>
@@ -19881,7 +19891,7 @@
     </row>
     <row r="295">
       <c r="A295" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B295" s="2" t="n">
         <v>442.187666137333</v>
@@ -19940,7 +19950,7 @@
     </row>
     <row r="296">
       <c r="A296" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B296" s="2" t="n">
         <v>390.12861551446</v>
@@ -19999,7 +20009,7 @@
     </row>
     <row r="297">
       <c r="A297" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B297" s="2" t="n">
         <v>397.333063871385</v>
@@ -20058,7 +20068,7 @@
     </row>
     <row r="298">
       <c r="A298" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B298" s="2" t="n">
         <v>411.227744528023</v>
@@ -20117,7 +20127,7 @@
     </row>
     <row r="299">
       <c r="A299" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B299" s="2" t="n">
         <v>378.080899652593</v>
@@ -20176,7 +20186,7 @@
     </row>
     <row r="300">
       <c r="A300" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B300" s="2" t="n">
         <v>394.838220618711</v>
@@ -20235,7 +20245,7 @@
     </row>
     <row r="301">
       <c r="A301" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B301" s="2" t="n">
         <v>422.671065824635</v>
@@ -20294,7 +20304,7 @@
     </row>
     <row r="302">
       <c r="A302" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B302" s="2" t="n">
         <v>421.347712921066</v>
@@ -20353,7 +20363,7 @@
     </row>
     <row r="303">
       <c r="A303" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B303" s="2" t="n">
         <v>403.896508596111</v>
@@ -20412,7 +20422,7 @@
     </row>
     <row r="304">
       <c r="A304" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B304" s="2" t="n">
         <v>352.586406411203</v>
@@ -20471,7 +20481,7 @@
     </row>
     <row r="305">
       <c r="A305" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B305" s="2" t="n">
         <v>377.504298767301</v>
@@ -20530,7 +20540,7 @@
     </row>
     <row r="306">
       <c r="A306" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B306" s="2" t="n">
         <v>414.953691139346</v>
@@ -20589,7 +20599,7 @@
     </row>
     <row r="307">
       <c r="A307" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B307" s="2" t="n">
         <v>471.236768995796</v>
@@ -20648,7 +20658,7 @@
     </row>
     <row r="308">
       <c r="A308" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B308" s="2" t="n">
         <v>431.457050866689</v>
@@ -20707,7 +20717,7 @@
     </row>
     <row r="309">
       <c r="A309" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B309" s="2" t="n">
         <v>433.004879917971</v>
@@ -20766,7 +20776,7 @@
     </row>
     <row r="310">
       <c r="A310" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B310" s="2" t="n">
         <v>441.549042990298</v>
@@ -20825,7 +20835,7 @@
     </row>
     <row r="311">
       <c r="A311" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B311" s="2" t="n">
         <v>419.232551781808</v>
@@ -20884,7 +20894,7 @@
     </row>
     <row r="312">
       <c r="A312" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B312" s="2" t="n">
         <v>425.781257296483</v>
@@ -20943,7 +20953,7 @@
     </row>
     <row r="313">
       <c r="A313" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B313" s="2" t="n">
         <v>426.691630423601</v>
@@ -21002,7 +21012,7 @@
     </row>
     <row r="314">
       <c r="A314" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B314" s="2" t="n">
         <v>427.568693202093</v>
@@ -21061,7 +21071,7 @@
     </row>
     <row r="315">
       <c r="A315" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B315" s="2" t="n">
         <v>410.213012430914</v>
@@ -21120,7 +21130,7 @@
     </row>
     <row r="316">
       <c r="A316" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B316" s="2" t="n">
         <v>410.591040989857</v>
@@ -21179,7 +21189,7 @@
     </row>
     <row r="317">
       <c r="A317" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B317" s="2" t="n">
         <v>391.130356114612</v>
@@ -21238,7 +21248,7 @@
     </row>
     <row r="318">
       <c r="A318" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B318" s="2" t="n">
         <v>480.781153834224</v>
@@ -21297,7 +21307,7 @@
     </row>
     <row r="319">
       <c r="A319" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B319" s="2" t="n">
         <v>515.146248104808</v>
@@ -21356,7 +21366,7 @@
     </row>
     <row r="320">
       <c r="A320" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B320" s="2" t="n">
         <v>420.149049692803</v>
@@ -21415,7 +21425,7 @@
     </row>
     <row r="321">
       <c r="A321" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B321" s="2" t="n">
         <v>446.556055385966</v>
@@ -21474,7 +21484,7 @@
     </row>
     <row r="322">
       <c r="A322" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B322" s="2" t="n">
         <v>418.017943433868</v>
@@ -21533,7 +21543,7 @@
     </row>
     <row r="323">
       <c r="A323" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B323" s="2" t="n">
         <v>403.925237772119</v>
@@ -21592,7 +21602,7 @@
     </row>
     <row r="324">
       <c r="A324" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B324" s="2" t="n">
         <v>394.816362544432</v>
@@ -21651,7 +21661,7 @@
     </row>
     <row r="325">
       <c r="A325" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="B325" s="2" t="n">
         <v>395.992789167532</v>
@@ -21710,7 +21720,7 @@
     </row>
     <row r="326">
       <c r="A326" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B326" s="2" t="n">
         <v>399.787184139496</v>
@@ -21769,7 +21779,7 @@
     </row>
     <row r="327">
       <c r="A327" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="B327" s="2" t="n">
         <v>397.05077242456</v>
@@ -21828,7 +21838,7 @@
     </row>
     <row r="328">
       <c r="A328" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B328" s="2" t="n">
         <v>343.598209612805</v>
@@ -21887,7 +21897,7 @@
     </row>
     <row r="329">
       <c r="A329" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="B329" s="2" t="n">
         <v>361.720712826645</v>
@@ -21946,7 +21956,7 @@
     </row>
     <row r="330">
       <c r="A330" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B330" s="2" t="n">
         <v>447.619639193651</v>
@@ -22005,7 +22015,7 @@
     </row>
     <row r="331">
       <c r="A331" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="B331" s="2" t="n">
         <v>442.973928376799</v>
@@ -22064,7 +22074,7 @@
     </row>
     <row r="332">
       <c r="A332" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B332" s="2" t="n">
         <v>393.891456074371</v>
@@ -22123,7 +22133,7 @@
     </row>
     <row r="333">
       <c r="A333" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="B333" s="2" t="n">
         <v>408.286312367396</v>
@@ -22182,7 +22192,7 @@
     </row>
     <row r="334">
       <c r="A334" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B334" s="2" t="n">
         <v>377.549028537073</v>
@@ -22241,7 +22251,7 @@
     </row>
     <row r="335">
       <c r="A335" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="B335" s="2" t="n">
         <v>372.186173989461</v>
@@ -22300,7 +22310,7 @@
     </row>
     <row r="336">
       <c r="A336" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B336" s="2" t="n">
         <v>375.893324759093</v>
@@ -22359,7 +22369,7 @@
     </row>
     <row r="337">
       <c r="A337" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="B337" s="2" t="n">
         <v>370.590384511402</v>
@@ -22418,7 +22428,7 @@
     </row>
     <row r="338">
       <c r="A338" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="B338" s="2" t="n">
         <v>367.29358914511</v>
@@ -22477,7 +22487,7 @@
     </row>
     <row r="339">
       <c r="A339" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="B339" s="2" t="n">
         <v>382.182928889282</v>
@@ -22536,7 +22546,7 @@
     </row>
     <row r="340">
       <c r="A340" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="B340" s="2" t="n">
         <v>303.840889594965</v>
@@ -22595,7 +22605,7 @@
     </row>
     <row r="341">
       <c r="A341" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="B341" s="2" t="n">
         <v>285.56255171414</v>
@@ -22654,7 +22664,7 @@
     </row>
     <row r="342">
       <c r="A342" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="B342" s="2" t="n">
         <v>356.365238336813</v>
@@ -22713,7 +22723,7 @@
     </row>
     <row r="343">
       <c r="A343" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="B343" s="2" t="n">
         <v>410.640659074934</v>
@@ -22772,7 +22782,7 @@
     </row>
     <row r="344">
       <c r="A344" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="B344" s="2" t="n">
         <v>370.603664328176</v>
@@ -22831,7 +22841,7 @@
     </row>
     <row r="345">
       <c r="A345" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="B345" s="2" t="n">
         <v>419.712266582932</v>
@@ -22890,7 +22900,7 @@
     </row>
     <row r="346">
       <c r="A346" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="B346" s="2" t="n">
         <v>390.302140847419</v>
@@ -22949,7 +22959,7 @@
     </row>
     <row r="347">
       <c r="A347" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="B347" s="2" t="n">
         <v>412.207748131389</v>
@@ -23008,7 +23018,7 @@
     </row>
     <row r="348">
       <c r="A348" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="B348" s="2" t="n">
         <v>415.477758601862</v>
@@ -23067,7 +23077,7 @@
     </row>
     <row r="349">
       <c r="A349" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="B349" s="2" t="n">
         <v>408.500143247877</v>
@@ -23126,7 +23136,7 @@
     </row>
     <row r="350">
       <c r="A350" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B350" s="2" t="n">
         <v>390.04781536087</v>
@@ -23185,7 +23195,7 @@
     </row>
     <row r="351">
       <c r="A351" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="B351" s="2" t="n">
         <v>401.954826908142</v>
@@ -23244,7 +23254,7 @@
     </row>
     <row r="352">
       <c r="A352" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="B352" s="2" t="n">
         <v>370.751762874357</v>
@@ -23303,7 +23313,7 @@
     </row>
     <row r="353">
       <c r="A353" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="B353" s="2" t="n">
         <v>399.074782831273</v>
@@ -23362,7 +23372,7 @@
     </row>
     <row r="354">
       <c r="A354" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="B354" s="2" t="n">
         <v>398.152959426753</v>
@@ -23421,7 +23431,7 @@
     </row>
     <row r="355">
       <c r="A355" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B355" s="2" t="n">
         <v>443.067701418994</v>
@@ -23480,7 +23490,7 @@
     </row>
     <row r="356">
       <c r="A356" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="B356" s="2" t="n">
         <v>384.950342884574</v>
@@ -23539,7 +23549,7 @@
     </row>
     <row r="357">
       <c r="A357" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="B357" s="2" t="n">
         <v>446.502460381261</v>
@@ -23598,7 +23608,7 @@
     </row>
     <row r="358">
       <c r="A358" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B358" s="2" t="n">
         <v>418.652096753782</v>
@@ -23657,7 +23667,7 @@
     </row>
     <row r="359">
       <c r="A359" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B359" s="2" t="n">
         <v>406.860841004746</v>
@@ -23716,7 +23726,7 @@
     </row>
     <row r="360">
       <c r="A360" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B360" s="2" t="n">
         <v>415.524634277786</v>
@@ -23775,7 +23785,7 @@
     </row>
     <row r="361">
       <c r="A361" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="B361" s="2" t="n">
         <v>444.851019235235</v>
@@ -23834,7 +23844,7 @@
     </row>
     <row r="362">
       <c r="A362" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="B362" s="2" t="n">
         <v>407.790757220666</v>
@@ -23893,7 +23903,7 @@
     </row>
     <row r="363">
       <c r="A363" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="B363" s="2" t="n">
         <v>429.747033158219</v>
@@ -23952,7 +23962,7 @@
     </row>
     <row r="364">
       <c r="A364" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B364" s="2" t="n">
         <v>373.827989263794</v>
@@ -24011,7 +24021,7 @@
     </row>
     <row r="365">
       <c r="A365" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="B365" s="2" t="n">
         <v>416.811209752702</v>
@@ -24070,7 +24080,7 @@
     </row>
     <row r="366">
       <c r="A366" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B366" s="2" t="n">
         <v>449.651413452699</v>
@@ -24129,7 +24139,7 @@
     </row>
     <row r="367">
       <c r="A367" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B367" s="2" t="n">
         <v>495.633745066193</v>
@@ -24188,7 +24198,7 @@
     </row>
     <row r="368">
       <c r="A368" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B368" s="2" t="n">
         <v>435.998195725037</v>
@@ -24247,7 +24257,7 @@
     </row>
     <row r="369">
       <c r="A369" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="B369" s="2" t="n">
         <v>427.87176151078</v>
@@ -24306,7 +24316,7 @@
     </row>
     <row r="370">
       <c r="A370" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="B370" s="2" t="n">
         <v>422.110452083367</v>
@@ -24365,7 +24375,7 @@
     </row>
     <row r="371">
       <c r="A371" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="B371" s="2" t="n">
         <v>430.736006197729</v>
@@ -24424,7 +24434,7 @@
     </row>
     <row r="372">
       <c r="A372" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="B372" s="2" t="n">
         <v>419.190064757897</v>
@@ -24483,7 +24493,7 @@
     </row>
     <row r="373">
       <c r="A373" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="B373" s="2" t="n">
         <v>433.445560748591</v>
@@ -24542,7 +24552,7 @@
     </row>
     <row r="374">
       <c r="A374" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="B374" s="2" t="n">
         <v>409.615933661514</v>
@@ -24601,7 +24611,7 @@
     </row>
     <row r="375">
       <c r="A375" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="B375" s="2" t="n">
         <v>401.471496620427</v>
@@ -24660,7 +24670,7 @@
     </row>
     <row r="376">
       <c r="A376" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B376" s="2" t="n">
         <v>370.533100679544</v>
@@ -24719,7 +24729,7 @@
     </row>
     <row r="377">
       <c r="A377" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="B377" s="2" t="n">
         <v>387.903826745362</v>
@@ -24778,7 +24788,7 @@
     </row>
     <row r="378">
       <c r="A378" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="B378" s="2" t="n">
         <v>429.2124706709</v>
@@ -24837,7 +24847,7 @@
     </row>
     <row r="379">
       <c r="A379" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="B379" s="2" t="n">
         <v>478.543630263215</v>
@@ -24896,7 +24906,7 @@
     </row>
     <row r="380">
       <c r="A380" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="B380" s="2" t="n">
         <v>420.914998041805</v>
@@ -24955,7 +24965,7 @@
     </row>
     <row r="381">
       <c r="A381" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="B381" s="2" t="n">
         <v>444.809876061346</v>
@@ -25014,7 +25024,7 @@
     </row>
     <row r="382">
       <c r="A382" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="B382" s="2" t="n">
         <v>415.088911327276</v>
@@ -25073,7 +25083,7 @@
     </row>
     <row r="383">
       <c r="A383" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="B383" s="2" t="n">
         <v>410.09148699683</v>
@@ -25132,7 +25142,7 @@
     </row>
     <row r="384">
       <c r="A384" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="B384" s="2" t="n">
         <v>380.158939972712</v>
@@ -25191,7 +25201,7 @@
     </row>
     <row r="385">
       <c r="A385" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B385" s="2" t="n">
         <v>355.180537349348</v>
@@ -25250,7 +25260,7 @@
     </row>
     <row r="386">
       <c r="A386" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="B386" s="2" t="n">
         <v>365.84893312039</v>
@@ -25309,7 +25319,7 @@
     </row>
     <row r="387">
       <c r="A387" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="B387" s="2" t="n">
         <v>359.732306003875</v>
@@ -25368,7 +25378,7 @@
     </row>
     <row r="388">
       <c r="A388" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="B388" s="2" t="n">
         <v>305.091802358158</v>
@@ -25427,7 +25437,7 @@
     </row>
     <row r="389">
       <c r="A389" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="B389" s="2" t="n">
         <v>325.524454975416</v>
@@ -25486,7 +25496,7 @@
     </row>
     <row r="390">
       <c r="A390" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="B390" s="2" t="n">
         <v>488.086102212039</v>
@@ -25545,7 +25555,7 @@
     </row>
     <row r="391">
       <c r="A391" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B391" s="2" t="n">
         <v>385.260609010283</v>
@@ -25604,7 +25614,7 @@
     </row>
     <row r="392">
       <c r="A392" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B392" s="2" t="n">
         <v>345.357533681744</v>
@@ -25663,7 +25673,7 @@
     </row>
     <row r="393">
       <c r="A393" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="B393" s="2" t="n">
         <v>371.015063022357</v>
@@ -25722,7 +25732,7 @@
     </row>
     <row r="394">
       <c r="A394" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="B394" s="2" t="n">
         <v>399.61836470486</v>
@@ -25781,7 +25791,7 @@
     </row>
     <row r="395">
       <c r="A395" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B395" s="2" t="n">
         <v>373.186587084923</v>
@@ -25840,7 +25850,7 @@
     </row>
     <row r="396">
       <c r="A396" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="B396" s="2" t="n">
         <v>380.666429367266</v>
@@ -25899,7 +25909,7 @@
     </row>
     <row r="397">
       <c r="A397" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="B397" s="2" t="n">
         <v>368.639057006452</v>
@@ -25958,7 +25968,7 @@
     </row>
     <row r="398">
       <c r="A398" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B398" s="2" t="n">
         <v>394.431143721451</v>
@@ -26017,7 +26027,7 @@
     </row>
     <row r="399">
       <c r="A399" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="B399" s="2" t="n">
         <v>429.041763486223</v>
@@ -26076,7 +26086,7 @@
     </row>
     <row r="400">
       <c r="A400" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="B400" s="2" t="n">
         <v>323.547109652471</v>
@@ -26135,7 +26145,7 @@
     </row>
     <row r="401">
       <c r="A401" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="B401" s="2" t="n">
         <v>346.455171979654</v>
@@ -26194,7 +26204,7 @@
     </row>
     <row r="402">
       <c r="A402" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B402" s="2" t="n">
         <v>408.362279347264</v>
@@ -26253,7 +26263,7 @@
     </row>
     <row r="403">
       <c r="A403" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="B403" s="2" t="n">
         <v>414.444146904842</v>
@@ -26312,7 +26322,7 @@
     </row>
     <row r="404">
       <c r="A404" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B404" s="2" t="n">
         <v>384.377482766837</v>
@@ -26371,7 +26381,7 @@
     </row>
     <row r="405">
       <c r="A405" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B405" s="2" t="n">
         <v>388.709602232659</v>
@@ -26430,7 +26440,7 @@
     </row>
     <row r="406">
       <c r="A406" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="B406" s="2" t="n">
         <v>379.496924729342</v>
@@ -26489,7 +26499,7 @@
     </row>
     <row r="407">
       <c r="A407" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="B407" s="2" t="n">
         <v>368.845737347648</v>
@@ -26548,7 +26558,7 @@
     </row>
     <row r="408">
       <c r="A408" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B408" s="2" t="n">
         <v>364.448206439434</v>
@@ -26607,7 +26617,7 @@
     </row>
     <row r="409">
       <c r="A409" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="B409" s="2" t="n">
         <v>380.711936423477</v>
@@ -26666,7 +26676,7 @@
     </row>
     <row r="410">
       <c r="A410" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="B410" s="2" t="n">
         <v>387.556406634348</v>
@@ -26725,7 +26735,7 @@
     </row>
     <row r="411">
       <c r="A411" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="B411" s="2" t="n">
         <v>409.454845651979</v>
@@ -26784,7 +26794,7 @@
     </row>
     <row r="412">
       <c r="A412" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="B412" s="2" t="n">
         <v>313.020367492984</v>
@@ -26843,7 +26853,7 @@
     </row>
     <row r="413">
       <c r="A413" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B413" s="2"/>
       <c r="C413" s="3" t="n">
@@ -26874,7 +26884,7 @@
     </row>
     <row r="414">
       <c r="A414" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="B414" s="2"/>
       <c r="C414" s="3" t="n">
@@ -26905,7 +26915,7 @@
     </row>
     <row r="415">
       <c r="A415" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="B415" s="2"/>
       <c r="C415" s="3" t="n">
@@ -26936,7 +26946,7 @@
     </row>
     <row r="416">
       <c r="A416" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="B416" s="2"/>
       <c r="C416" s="3" t="n">
@@ -26967,7 +26977,7 @@
     </row>
     <row r="417">
       <c r="A417" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="B417" s="2"/>
       <c r="C417" s="3" t="n">
@@ -26998,7 +27008,7 @@
     </row>
     <row r="418">
       <c r="A418" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="B418" s="2"/>
       <c r="C418" s="3" t="n">
@@ -27029,7 +27039,7 @@
     </row>
     <row r="419">
       <c r="A419" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="B419" s="2"/>
       <c r="C419" s="3" t="n">
@@ -27060,7 +27070,7 @@
     </row>
     <row r="420">
       <c r="A420" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B420" s="2"/>
       <c r="C420" s="3" t="n">
@@ -27091,7 +27101,7 @@
     </row>
     <row r="421">
       <c r="A421" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="B421" s="2"/>
       <c r="C421" s="3" t="n">
@@ -27122,7 +27132,7 @@
     </row>
     <row r="422">
       <c r="A422" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="B422" s="2"/>
       <c r="C422" s="3" t="n">
@@ -27153,7 +27163,7 @@
     </row>
     <row r="423">
       <c r="A423" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="B423" s="2"/>
       <c r="C423" s="3" t="n">
@@ -27184,7 +27194,7 @@
     </row>
     <row r="424">
       <c r="A424" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="B424" s="2"/>
       <c r="C424" s="3" t="n">
@@ -27215,7 +27225,7 @@
     </row>
     <row r="425">
       <c r="A425" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="B425" s="2"/>
       <c r="C425" s="3"/>
@@ -27238,7 +27248,7 @@
     </row>
     <row r="426">
       <c r="A426" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="B426" s="2"/>
       <c r="C426" s="3"/>
@@ -27261,7 +27271,7 @@
     </row>
     <row r="427">
       <c r="A427" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="B427" s="2"/>
       <c r="C427" s="3"/>
@@ -27284,7 +27294,7 @@
     </row>
     <row r="428">
       <c r="A428" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B428" s="2"/>
       <c r="C428" s="3"/>
@@ -27307,7 +27317,7 @@
     </row>
     <row r="429">
       <c r="A429" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="B429" s="2"/>
       <c r="C429" s="3"/>
@@ -27330,7 +27340,7 @@
     </row>
     <row r="430">
       <c r="A430" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="B430" s="2"/>
       <c r="C430" s="3"/>
@@ -27353,7 +27363,7 @@
     </row>
     <row r="431">
       <c r="A431" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="B431" s="2"/>
       <c r="C431" s="3"/>
@@ -27376,7 +27386,7 @@
     </row>
     <row r="432">
       <c r="A432" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="B432" s="2"/>
       <c r="C432" s="3"/>
@@ -27399,7 +27409,7 @@
     </row>
     <row r="433">
       <c r="A433" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="B433" s="2"/>
       <c r="C433" s="3"/>
@@ -27422,7 +27432,7 @@
     </row>
     <row r="434">
       <c r="A434" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="B434" s="2"/>
       <c r="C434" s="3"/>
@@ -27445,7 +27455,7 @@
     </row>
     <row r="435">
       <c r="A435" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="B435" s="2"/>
       <c r="C435" s="3"/>
@@ -27468,7 +27478,7 @@
     </row>
     <row r="436">
       <c r="A436" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="B436" s="2"/>
       <c r="C436" s="3"/>
@@ -27491,7 +27501,7 @@
     </row>
     <row r="437">
       <c r="A437" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="B437" s="2"/>
       <c r="C437" s="3"/>
@@ -27514,7 +27524,7 @@
     </row>
     <row r="438">
       <c r="A438" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="B438" s="2"/>
       <c r="C438" s="3"/>
@@ -27537,7 +27547,7 @@
     </row>
     <row r="439">
       <c r="A439" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="B439" s="2"/>
       <c r="C439" s="3"/>
@@ -27560,7 +27570,7 @@
     </row>
     <row r="440">
       <c r="A440" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="B440" s="2"/>
       <c r="C440" s="3"/>
@@ -27583,7 +27593,7 @@
     </row>
     <row r="441">
       <c r="A441" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="B441" s="2"/>
       <c r="C441" s="3"/>
@@ -27606,7 +27616,7 @@
     </row>
     <row r="442">
       <c r="A442" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="B442" s="2"/>
       <c r="C442" s="3"/>
@@ -27629,7 +27639,7 @@
     </row>
     <row r="443">
       <c r="A443" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="B443" s="2"/>
       <c r="C443" s="3"/>
@@ -27652,7 +27662,7 @@
     </row>
     <row r="444">
       <c r="A444" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="B444" s="2"/>
       <c r="C444" s="3"/>
@@ -27675,7 +27685,7 @@
     </row>
     <row r="445">
       <c r="A445" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="B445" s="2"/>
       <c r="C445" s="3"/>
@@ -27698,7 +27708,7 @@
     </row>
     <row r="446">
       <c r="A446" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="B446" s="2"/>
       <c r="C446" s="3"/>
@@ -27721,7 +27731,7 @@
     </row>
     <row r="447">
       <c r="A447" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="B447" s="2"/>
       <c r="C447" s="3"/>
@@ -27744,7 +27754,7 @@
     </row>
     <row r="448">
       <c r="A448" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="B448" s="2"/>
       <c r="C448" s="3"/>
@@ -27767,7 +27777,7 @@
     </row>
     <row r="449">
       <c r="A449" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="B449" s="2"/>
       <c r="C449" s="3"/>
@@ -27790,7 +27800,7 @@
     </row>
     <row r="450">
       <c r="A450" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="B450" s="2"/>
       <c r="C450" s="3"/>
@@ -27813,7 +27823,7 @@
     </row>
     <row r="451">
       <c r="A451" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="B451" s="2"/>
       <c r="C451" s="3"/>
@@ -27836,7 +27846,7 @@
     </row>
     <row r="452">
       <c r="A452" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="B452" s="2"/>
       <c r="C452" s="3"/>
@@ -27859,7 +27869,7 @@
     </row>
     <row r="453">
       <c r="A453" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="B453" s="2"/>
       <c r="C453" s="3"/>
@@ -27882,7 +27892,7 @@
     </row>
     <row r="454">
       <c r="A454" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="B454" s="2"/>
       <c r="C454" s="3"/>
@@ -27905,7 +27915,7 @@
     </row>
     <row r="455">
       <c r="A455" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="B455" s="2"/>
       <c r="C455" s="3"/>
@@ -27928,7 +27938,7 @@
     </row>
     <row r="456">
       <c r="A456" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="B456" s="2"/>
       <c r="C456" s="3"/>
@@ -27951,7 +27961,7 @@
     </row>
     <row r="457">
       <c r="A457" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="B457" s="2"/>
       <c r="C457" s="3"/>
@@ -27974,7 +27984,7 @@
     </row>
     <row r="458">
       <c r="A458" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="B458" s="2"/>
       <c r="C458" s="3"/>
@@ -27997,7 +28007,7 @@
     </row>
     <row r="459">
       <c r="A459" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="B459" s="2"/>
       <c r="C459" s="3"/>
@@ -28020,7 +28030,7 @@
     </row>
     <row r="460">
       <c r="A460" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="B460" s="2"/>
       <c r="C460" s="3"/>
@@ -28043,7 +28053,7 @@
     </row>
     <row r="461">
       <c r="A461" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="B461" s="2"/>
       <c r="C461" s="3"/>
@@ -28066,7 +28076,7 @@
     </row>
     <row r="462">
       <c r="A462" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="B462" s="2"/>
       <c r="C462" s="3"/>
@@ -28089,7 +28099,7 @@
     </row>
     <row r="463">
       <c r="A463" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="B463" s="2"/>
       <c r="C463" s="3"/>
@@ -28112,7 +28122,7 @@
     </row>
     <row r="464">
       <c r="A464" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="B464" s="2"/>
       <c r="C464" s="3"/>
@@ -28135,7 +28145,7 @@
     </row>
     <row r="465">
       <c r="A465" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="B465" s="2"/>
       <c r="C465" s="3"/>
@@ -28158,7 +28168,7 @@
     </row>
     <row r="466">
       <c r="A466" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="B466" s="2"/>
       <c r="C466" s="3"/>
@@ -28181,7 +28191,7 @@
     </row>
     <row r="467">
       <c r="A467" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="B467" s="2"/>
       <c r="C467" s="3"/>
@@ -28204,7 +28214,7 @@
     </row>
     <row r="468">
       <c r="A468" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="B468" s="2"/>
       <c r="C468" s="3"/>
@@ -28227,7 +28237,7 @@
     </row>
     <row r="469">
       <c r="A469" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="B469" s="2"/>
       <c r="C469" s="3"/>
@@ -28261,97 +28271,97 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
     </row>
   </sheetData>
@@ -28375,7 +28385,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -28385,160 +28395,160 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>0.137491082967171</v>
+        <v>0.136107350155359</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.164263395700548</v>
+        <v>0.162601614946108</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.194180838142898</v>
+        <v>0.192665360117761</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.216957414207872</v>
+        <v>0.216222333256039</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.23198583485394</v>
+        <v>0.232668182014414</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.287955626610621</v>
+        <v>0.28790874610718</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.342562006011485</v>
+        <v>0.341526869222225</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.419109102966695</v>
+        <v>0.419018665246809</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.592728983090691</v>
+        <v>0.592558065563799</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.681640615226608</v>
+        <v>0.680782880624759</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.54486223581441</v>
+        <v>0.544740982052114</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.406556247451318</v>
+        <v>0.407528869463841</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.360097128876648</v>
+        <v>0.361886652029656</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.306534556100409</v>
+        <v>0.308951348086236</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.267758034795071</v>
+        <v>0.269577126091802</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.25711858461795</v>
+        <v>0.257972372783113</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>0.224315373413365</v>
+        <v>0.225561165275108</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>0.178990870137532</v>
+        <v>0.180650962852167</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>0.138644244474717</v>
+        <v>0.139032647584844</v>
       </c>
     </row>
     <row r="24">

</xml_diff>

<commit_message>
Corrida | SFE-RTT | 2026-08-21 13:12:41.591621
</commit_message>
<xml_diff>
--- a/indicadores/SFE-RTT_out.xlsx
+++ b/indicadores/SFE-RTT_out.xlsx
@@ -104,13 +104,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">31/07/2026</t>
+    <t xml:space="preserve">21/08/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">pcohan</t>
+    <t xml:space="preserve">fleiva</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -2253,7 +2253,7 @@
       <c r="B11"/>
       <c r="C11"/>
       <c r="D11" t="n">
-        <v>0.695155392149454</v>
+        <v>0.696135836498929</v>
       </c>
       <c r="E11"/>
       <c r="F11"/>
@@ -2311,7 +2311,7 @@
       <c r="B15"/>
       <c r="C15"/>
       <c r="D15" t="n">
-        <v>0.483241019234461</v>
+        <v>0.484605102858062</v>
       </c>
       <c r="E15"/>
       <c r="F15"/>
@@ -2381,7 +2381,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.00000000148173064879474</v>
+        <v>0.00000000101002342018422</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -2411,7 +2411,7 @@
       <c r="B22"/>
       <c r="C22"/>
       <c r="D22" t="n">
-        <v>0.0000089995409241783</v>
+        <v>0.00000401989369496798</v>
       </c>
       <c r="E22"/>
       <c r="F22"/>
@@ -28476,7 +28476,7 @@
         <v>540</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>0.171119902078616</v>
+        <v>0.17090346942517</v>
       </c>
     </row>
     <row r="6">
@@ -28484,7 +28484,7 @@
         <v>541</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.173534137786483</v>
+        <v>0.173577736720583</v>
       </c>
     </row>
     <row r="7">
@@ -28492,7 +28492,7 @@
         <v>542</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.169685750510732</v>
+        <v>0.170103064455823</v>
       </c>
     </row>
     <row r="8">
@@ -28500,7 +28500,7 @@
         <v>543</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.183958951646156</v>
+        <v>0.184685794981476</v>
       </c>
     </row>
     <row r="9">
@@ -28508,7 +28508,7 @@
         <v>544</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.186923182793551</v>
+        <v>0.187464808189498</v>
       </c>
     </row>
     <row r="10">
@@ -28516,7 +28516,7 @@
         <v>545</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.255929093704953</v>
+        <v>0.256143707729641</v>
       </c>
     </row>
     <row r="11">
@@ -28524,7 +28524,7 @@
         <v>546</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.344997504597351</v>
+        <v>0.345416921158953</v>
       </c>
     </row>
     <row r="12">
@@ -28532,7 +28532,7 @@
         <v>547</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.441148190519249</v>
+        <v>0.441603001099644</v>
       </c>
     </row>
     <row r="13">
@@ -28540,7 +28540,7 @@
         <v>548</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.612976737198136</v>
+        <v>0.613450102560706</v>
       </c>
     </row>
     <row r="14">
@@ -28548,7 +28548,7 @@
         <v>549</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.695155392149454</v>
+        <v>0.696135836498929</v>
       </c>
     </row>
     <row r="15">
@@ -28556,7 +28556,7 @@
         <v>550</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.56856734556109</v>
+        <v>0.56934097008359</v>
       </c>
     </row>
     <row r="16">
@@ -28564,7 +28564,7 @@
         <v>551</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.431618111717723</v>
+        <v>0.431429047288774</v>
       </c>
     </row>
     <row r="17">
@@ -28572,7 +28572,7 @@
         <v>552</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.360679792084339</v>
+        <v>0.360457080183058</v>
       </c>
     </row>
     <row r="18">
@@ -28580,7 +28580,7 @@
         <v>553</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.306839890313392</v>
+        <v>0.307348995321574</v>
       </c>
     </row>
     <row r="19">
@@ -28588,7 +28588,7 @@
         <v>554</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.263713799729729</v>
+        <v>0.264403898590981</v>
       </c>
     </row>
     <row r="20">
@@ -28596,7 +28596,7 @@
         <v>555</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.240531676266438</v>
+        <v>0.239861293702612</v>
       </c>
     </row>
     <row r="21">
@@ -28604,7 +28604,7 @@
         <v>556</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>0.227401345145639</v>
+        <v>0.226169808356571</v>
       </c>
     </row>
     <row r="22">
@@ -28612,7 +28612,7 @@
         <v>557</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>0.192874010969585</v>
+        <v>0.192886512969933</v>
       </c>
     </row>
     <row r="23">
@@ -28620,7 +28620,7 @@
         <v>558</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>0.138836594515647</v>
+        <v>0.139303132255753</v>
       </c>
     </row>
     <row r="24">

</xml_diff>